<commit_message>
update / feature: plan excel
Implemento de formatação de planilha de comissão com duas casas decimais e última linha (total) em negrito.
</commit_message>
<xml_diff>
--- a/Relatorio_Comissao_Gerencial.xlsx
+++ b/Relatorio_Comissao_Gerencial.xlsx
@@ -55,11 +55,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -491,34 +493,34 @@
           <t>2026-03-01</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>25.884</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.884</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.884</v>
-      </c>
-      <c r="E2" t="n">
-        <v>25.884</v>
-      </c>
-      <c r="F2" t="n">
-        <v>25.884</v>
-      </c>
-      <c r="G2" t="n">
-        <v>25.884</v>
-      </c>
-      <c r="H2" t="n">
-        <v>25.884</v>
-      </c>
-      <c r="I2" t="n">
-        <v>25.884</v>
-      </c>
-      <c r="J2" t="n">
-        <v>25.884</v>
-      </c>
-      <c r="K2" t="n">
+      <c r="B2" s="2" t="n">
+        <v>25.884</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>25.884</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>25.884</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>25.884</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>25.884</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>25.884</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>25.884</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>25.884</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>25.884</v>
+      </c>
+      <c r="K2" s="2" t="n">
         <v>25.884</v>
       </c>
     </row>
@@ -528,34 +530,34 @@
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>12.28</v>
-      </c>
-      <c r="C3" t="n">
-        <v>12.28</v>
-      </c>
-      <c r="D3" t="n">
-        <v>12.28</v>
-      </c>
-      <c r="E3" t="n">
-        <v>12.28</v>
-      </c>
-      <c r="F3" t="n">
-        <v>12.28</v>
-      </c>
-      <c r="G3" t="n">
-        <v>12.28</v>
-      </c>
-      <c r="H3" t="n">
-        <v>12.28</v>
-      </c>
-      <c r="I3" t="n">
-        <v>12.28</v>
-      </c>
-      <c r="J3" t="n">
-        <v>12.28</v>
-      </c>
-      <c r="K3" t="n">
+      <c r="B3" s="2" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="K3" s="2" t="n">
         <v>12.28</v>
       </c>
     </row>
@@ -565,34 +567,34 @@
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>22.552</v>
-      </c>
-      <c r="C4" t="n">
-        <v>22.552</v>
-      </c>
-      <c r="D4" t="n">
-        <v>22.552</v>
-      </c>
-      <c r="E4" t="n">
-        <v>22.552</v>
-      </c>
-      <c r="F4" t="n">
-        <v>22.552</v>
-      </c>
-      <c r="G4" t="n">
-        <v>22.552</v>
-      </c>
-      <c r="H4" t="n">
-        <v>22.552</v>
-      </c>
-      <c r="I4" t="n">
-        <v>22.552</v>
-      </c>
-      <c r="J4" t="n">
-        <v>22.552</v>
-      </c>
-      <c r="K4" t="n">
+      <c r="B4" s="2" t="n">
+        <v>22.552</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>22.552</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>22.552</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>22.552</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>22.552</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>22.552</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>22.552</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>22.552</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>22.552</v>
+      </c>
+      <c r="K4" s="2" t="n">
         <v>22.552</v>
       </c>
     </row>
@@ -602,34 +604,34 @@
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>17.64</v>
-      </c>
-      <c r="C5" t="n">
-        <v>17.64</v>
-      </c>
-      <c r="D5" t="n">
-        <v>17.64</v>
-      </c>
-      <c r="E5" t="n">
-        <v>17.64</v>
-      </c>
-      <c r="F5" t="n">
-        <v>17.64</v>
-      </c>
-      <c r="G5" t="n">
-        <v>17.64</v>
-      </c>
-      <c r="H5" t="n">
-        <v>17.64</v>
-      </c>
-      <c r="I5" t="n">
-        <v>17.64</v>
-      </c>
-      <c r="J5" t="n">
-        <v>17.64</v>
-      </c>
-      <c r="K5" t="n">
+      <c r="B5" s="2" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="K5" s="2" t="n">
         <v>17.64</v>
       </c>
     </row>
@@ -639,34 +641,34 @@
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>13.752</v>
-      </c>
-      <c r="C6" t="n">
-        <v>13.752</v>
-      </c>
-      <c r="D6" t="n">
-        <v>13.752</v>
-      </c>
-      <c r="E6" t="n">
-        <v>13.752</v>
-      </c>
-      <c r="F6" t="n">
-        <v>13.752</v>
-      </c>
-      <c r="G6" t="n">
-        <v>13.752</v>
-      </c>
-      <c r="H6" t="n">
-        <v>13.752</v>
-      </c>
-      <c r="I6" t="n">
-        <v>13.752</v>
-      </c>
-      <c r="J6" t="n">
-        <v>13.752</v>
-      </c>
-      <c r="K6" t="n">
+      <c r="B6" s="2" t="n">
+        <v>13.752</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>13.752</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>13.752</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>13.752</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>13.752</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>13.752</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>13.752</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>13.752</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>13.752</v>
+      </c>
+      <c r="K6" s="2" t="n">
         <v>13.752</v>
       </c>
     </row>
@@ -676,34 +678,34 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>92.10799999999999</v>
-      </c>
-      <c r="C7" t="n">
-        <v>92.10799999999999</v>
-      </c>
-      <c r="D7" t="n">
-        <v>92.10799999999999</v>
-      </c>
-      <c r="E7" t="n">
-        <v>92.10799999999999</v>
-      </c>
-      <c r="F7" t="n">
-        <v>92.10799999999999</v>
-      </c>
-      <c r="G7" t="n">
-        <v>92.10799999999999</v>
-      </c>
-      <c r="H7" t="n">
-        <v>92.10799999999999</v>
-      </c>
-      <c r="I7" t="n">
-        <v>92.10799999999999</v>
-      </c>
-      <c r="J7" t="n">
-        <v>92.10799999999999</v>
-      </c>
-      <c r="K7" t="n">
+      <c r="B7" s="3" t="n">
+        <v>92.10799999999999</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>92.10799999999999</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>92.10799999999999</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>92.10799999999999</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>92.10799999999999</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>92.10799999999999</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>92.10799999999999</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>92.10799999999999</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>92.10799999999999</v>
+      </c>
+      <c r="K7" s="3" t="n">
         <v>92.10799999999999</v>
       </c>
     </row>

</xml_diff>